<commit_message>
Improve car specs and telegram post template
</commit_message>
<xml_diff>
--- a/app/data/korex_latest.xlsx
+++ b/app/data/korex_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y22"/>
+  <dimension ref="A1:AD22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,45 +499,70 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>fuelConsumption</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>acceleration0100</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>maxSpeed</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>maxPowerKw</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>maxTorqueNm</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>torqueNm</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
         <is>
           <t>dimensions</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>engineVolume</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
         <is>
           <t>wheelbase</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>seats</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>fuelTankVolume</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>tireSize</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>images</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>remoteImages</t>
         </is>
@@ -623,40 +648,73 @@
           <t>Передний привод</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>(кВт)</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>100</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr">
         <is>
           <t>["/uploads/cars/1/1.webp", "/uploads/cars/1/2.webp", "/uploads/cars/1/3.webp", "/uploads/cars/1/4.webp"]</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/83356300/1775240582.6787.webp", "https://cn2.pa-server.ru/img/19/2026/04/83356300/1775240584.2652.webp", "https://cn2.pa-server.ru/img/19/2026/04/83356300/1775240585.3933.webp", "https://cn2.pa-server.ru/img/19/2026/04/83356300/1775240586.6656.webp", "https://cn2.pa-server.ru/img/19/2026/04/83356300/1775240587.8374.webp", "https://cn2.pa-server.ru/img/19/2026/04/83356300/1775240588.9285.webp", "https://cn2.pa-server.ru/img/19/2026/04/83356300/1775240590.1843.webp", "https://cn2.pa-server.ru/img/19/2026/04/83356300/1775240591.1193.webp", "https://cn2.pa-server.ru/img/19/2026/04/83356300/1775240592.1774.webp"]</t>
         </is>
@@ -742,40 +800,73 @@
           <t>Передний привод</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>(кВт)</t>
+          <t>5.8</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr">
         <is>
           <t>["/uploads/cars/2/1.webp", "/uploads/cars/2/2.webp", "/uploads/cars/2/3.webp", "/uploads/cars/2/4.webp"]</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467022.8412.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467024.171.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467025.4411.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467026.9505.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467028.5202.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467031.0285.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467033.1602.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467034.4444.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467035.8928.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467037.1592.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467038.3991.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467039.2013.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467040.4828.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467041.7103.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467042.8958.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467044.0818.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467045.1429.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467046.1647.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467048.0763.webp", "https://cn2.pa-server.ru/img/19/2026/04/83854368/1775467049.4708.webp"]</t>
         </is>
@@ -862,39 +953,64 @@
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr"/>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>4565*1821*1620</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>2780</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>["/uploads/cars/3/1.webp", "/uploads/cars/3/2.webp", "/uploads/cars/3/3.webp", "/uploads/cars/3/4.webp"]</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795522.5921.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795523.4385.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795524.3466.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795525.3023.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795526.1655.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795527.4482.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795528.4265.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795529.4986.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795530.5106.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795531.49.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795532.4745.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795533.6078.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795534.5832.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795535.5515.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795536.4098.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795537.2178.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795538.0256.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795539.3341.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795540.5363.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795541.4337.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795542.2944.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795543.5939.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795544.5338.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795545.345.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795546.0732.webp", "https://cn2.pa-server.ru/img/19/2026/04/84680391/1775795546.8035.webp"]</t>
         </is>
@@ -980,40 +1096,73 @@
           <t>Передний привод</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>(кВт)</t>
+          <t>5.8</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr">
         <is>
           <t>["/uploads/cars/4/1.webp", "/uploads/cars/4/2.webp", "/uploads/cars/4/3.webp", "/uploads/cars/4/4.webp"]</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/84850133/1775882822.7281.webp", "https://cn2.pa-server.ru/img/19/2026/04/84850133/1775882823.7049.webp", "https://cn2.pa-server.ru/img/19/2026/04/84850133/1775882824.8993.webp", "https://cn2.pa-server.ru/img/19/2026/04/84850133/1775882825.8977.webp", "https://cn2.pa-server.ru/img/19/2026/04/84850133/1775882826.9914.webp", "https://cn2.pa-server.ru/img/19/2026/04/84850133/1775882828.8425.webp", "https://cn2.pa-server.ru/img/19/2026/04/84850133/1775882829.9365.webp", "https://cn2.pa-server.ru/img/19/2026/04/84850133/1775882830.74.webp", "https://cn2.pa-server.ru/img/19/2026/04/84850133/1775882831.4858.webp", "https://cn2.pa-server.ru/img/19/2026/04/84850133/1775882832.4338.webp"]</t>
         </is>
@@ -1100,39 +1249,64 @@
         </is>
       </c>
       <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr">
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr">
         <is>
           <t>["/uploads/cars/5/1.webp", "/uploads/cars/5/2.webp", "/uploads/cars/5/3.webp", "/uploads/cars/5/4.webp"]</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884022.6416.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884023.4839.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884024.2452.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884025.0722.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884025.7904.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884026.754.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884027.4674.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884028.1523.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884028.9918.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884030.531.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884031.7703.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884032.7432.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884033.9102.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884035.0485.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884036.3523.webp", "https://cn2.pa-server.ru/img/19/2026/04/84851710/1775884037.59.webp"]</t>
         </is>
@@ -1218,40 +1392,73 @@
           <t>Передний привод</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>(кВт)</t>
+          <t>5.8</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr">
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr">
         <is>
           <t>["/uploads/cars/6/1.webp", "/uploads/cars/6/2.webp", "/uploads/cars/6/3.webp", "/uploads/cars/6/4.webp"]</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="AD7" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389523.0968.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389524.0815.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389525.0279.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389526.1884.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389527.1717.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389528.1713.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389529.1587.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389529.963.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389530.8636.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389532.4492.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389533.3464.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389534.672.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389535.601.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389536.3457.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389537.5315.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389538.5232.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389539.6943.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389540.7889.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389543.122.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839661/1776389544.1092.webp"]</t>
         </is>
@@ -1338,39 +1545,64 @@
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr">
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr">
         <is>
           <t>["/uploads/cars/7/1.webp", "/uploads/cars/7/2.webp", "/uploads/cars/7/3.webp", "/uploads/cars/7/4.webp"]</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389763.6037.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389765.4066.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389766.4058.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389767.6292.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389768.9342.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389770.1762.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389771.0883.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389772.2491.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389773.4153.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389774.7909.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389776.4314.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389777.3586.webp", "https://cn2.pa-server.ru/img/19/2026/04/85839761/1776389778.675.webp"]</t>
         </is>
@@ -1456,40 +1688,73 @@
           <t>Передний привод</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>(кВт)</t>
+          <t>5.8</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr">
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr">
         <is>
           <t>["/uploads/cars/8/1.webp", "/uploads/cars/8/2.webp", "/uploads/cars/8/3.webp", "/uploads/cars/8/4.webp"]</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="AD9" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391622.9177.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391623.8902.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391624.6052.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391625.5359.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391626.6122.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391627.8774.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391628.9405.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391630.1704.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391631.1331.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391632.1679.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391633.1036.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391634.4348.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391635.8274.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391636.92.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391637.9409.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391639.0403.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391640.0177.webp", "https://cn2.pa-server.ru/img/19/2026/04/85843180/1776391641.3209.webp"]</t>
         </is>
@@ -1576,39 +1841,64 @@
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr">
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr">
         <is>
           <t>["/uploads/cars/9/1.webp", "/uploads/cars/9/2.webp", "/uploads/cars/9/3.webp", "/uploads/cars/9/4.webp"]</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
+      <c r="AD10" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499803.1896.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499804.1679.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499805.0117.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499805.938.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499807.7975.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499808.8924.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499809.9599.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499811.0511.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499811.8797.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499812.9296.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499814.235.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499815.3549.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499816.8301.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499818.1838.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499819.1149.webp", "https://cn2.pa-server.ru/img/19/2026/04/86068057/1776499820.1094.webp"]</t>
         </is>
@@ -1695,39 +1985,64 @@
         </is>
       </c>
       <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr"/>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>4565*1821*1620</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>2780</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr">
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr">
         <is>
           <t>["/uploads/cars/10/1.webp"]</t>
         </is>
       </c>
-      <c r="Y11" t="inlineStr">
+      <c r="AD11" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950282.5339.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950283.8095.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950286.6178.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950287.8212.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950288.9669.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950289.9928.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950291.0634.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950296.5834.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950297.4458.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950298.6521.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950299.7621.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950300.7244.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950301.7542.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950303.1062.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950304.5573.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950305.7211.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950306.9552.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950307.9678.webp", "https://cn2.pa-server.ru/img/19/2026/04/86680456/1776950309.3269.webp"]</t>
         </is>
@@ -1814,39 +2129,64 @@
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr">
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr">
         <is>
           <t>["/uploads/cars/11/1.webp", "/uploads/cars/11/2.webp", "/uploads/cars/11/3.webp", "/uploads/cars/11/4.webp"]</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="AD12" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244828.5049.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244834.7812.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244840.3834.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244841.2606.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244847.6851.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244851.1964.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244852.6853.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244853.84.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244855.8758.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244857.7816.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244863.109.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244865.3057.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244870.305.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244874.3127.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244886.3896.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244888.643.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244889.67.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244897.8163.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244904.1736.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244905.6084.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244906.3097.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244907.5895.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244908.4484.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244909.4056.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244910.766.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244911.4444.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244912.7633.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244913.7057.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244914.5636.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244915.2639.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244922.0691.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244923.3506.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244924.0828.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244925.4558.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857852/1777244926.5543.webp"]</t>
         </is>
@@ -1932,40 +2272,73 @@
           <t>Передний привод</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>(кВт)</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>100</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr">
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr">
         <is>
           <t>["/uploads/cars/12/1.webp", "/uploads/cars/12/2.webp", "/uploads/cars/12/3.webp", "/uploads/cars/12/4.webp"]</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="AD13" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244890.4323.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244895.8655.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244896.9078.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244898.2357.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244903.6859.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244904.6478.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244906.009.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244908.7871.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244910.5731.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244911.4275.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244912.5667.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244913.7241.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244916.279.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244921.2316.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244922.8557.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244924.8523.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244926.0717.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857873/1777244927.4872.webp"]</t>
         </is>
@@ -2052,39 +2425,64 @@
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr">
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr">
         <is>
           <t>["/uploads/cars/13/1.webp", "/uploads/cars/13/2.webp", "/uploads/cars/13/3.webp", "/uploads/cars/13/4.webp"]</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
+      <c r="AD14" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244947.9099.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244954.0732.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244960.8362.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244967.9159.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244970.0177.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244974.3282.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244975.2027.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244976.3725.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244979.5784.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244980.9543.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244986.94.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244988.483.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244989.9008.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244994.6408.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244996.8898.webp", "https://cn2.pa-server.ru/img/19/2026/04/86857886/1777244998.2705.webp"]</t>
         </is>
@@ -2170,40 +2568,73 @@
           <t>Передний привод</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>(кВт)</t>
+          <t>5.8</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr">
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr">
         <is>
           <t>["/uploads/cars/14/1.webp", "/uploads/cars/14/2.webp", "/uploads/cars/14/3.webp", "/uploads/cars/14/4.webp"]</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="AD15" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245069.3321.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245074.9927.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245082.1594.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245083.4881.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245087.8166.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245088.7771.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245091.9096.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245099.5994.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245100.5653.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245101.4765.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245109.2062.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858435/1777245111.5725.webp"]</t>
         </is>
@@ -2290,39 +2721,64 @@
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr">
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr">
         <is>
           <t>["/uploads/cars/15/1.webp", "/uploads/cars/15/2.webp", "/uploads/cars/15/3.webp", "/uploads/cars/15/4.webp"]</t>
         </is>
       </c>
-      <c r="Y16" t="inlineStr">
+      <c r="AD16" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245067.3152.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245069.1928.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245074.993.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245081.1921.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245082.8505.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245086.1326.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245087.2948.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245089.9416.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245091.4904.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245097.5779.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245100.98.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245107.3955.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245108.3012.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245109.3329.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245111.0845.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245114.2095.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245119.6438.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245120.6198.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245121.9838.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245127.8575.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245130.0711.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245134.9381.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245140.5921.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245143.2232.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245144.2948.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245145.3925.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245151.3951.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245152.4089.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245153.3888.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245154.4314.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245155.3325.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245156.1393.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245157.2617.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245158.3331.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245159.4981.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245160.5324.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245161.5985.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245162.4789.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858445/1777245163.6478.webp"]</t>
         </is>
@@ -2409,39 +2865,64 @@
         </is>
       </c>
       <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr">
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr">
         <is>
           <t>["/uploads/cars/16/1.webp", "/uploads/cars/16/2.webp", "/uploads/cars/16/3.webp", "/uploads/cars/16/4.webp"]</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr">
+      <c r="AD17" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/86858469/1777245067.347.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858469/1777245070.5551.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858469/1777245075.8851.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858469/1777245081.5473.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858469/1777245083.9222.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858469/1777245085.2107.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858469/1777245087.5521.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858469/1777245088.5635.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858469/1777245089.4906.webp"]</t>
         </is>
@@ -2528,39 +3009,64 @@
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>4462*1803*1446</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>2670</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr">
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr">
         <is>
           <t>["/uploads/cars/17/1.webp", "/uploads/cars/17/2.webp", "/uploads/cars/17/3.webp", "/uploads/cars/17/4.webp"]</t>
         </is>
       </c>
-      <c r="Y18" t="inlineStr">
+      <c r="AD18" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245308.3192.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245311.2741.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245321.8934.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245329.7271.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245335.6573.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245339.2973.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245343.4526.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245347.0125.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245351.2533.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245353.0763.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245354.1224.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245360.435.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245361.493.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245363.2519.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245364.8581.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245370.5498.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245371.8175.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245377.247.webp", "https://cn2.pa-server.ru/img/19/2026/04/86858713/1777245383.3265.webp"]</t>
         </is>
@@ -2646,40 +3152,73 @@
           <t>Передний привод</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>6.9</t>
+        </is>
+      </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>(кВт)</t>
+          <t>6.9</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr"/>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>4565*1821*1620</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>2780</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr">
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr">
         <is>
           <t>["/uploads/cars/18/1.webp"]</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
+      <c r="AD19" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618206.7949.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618207.9903.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618208.9328.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618210.3289.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618211.5157.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618212.6296.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618214.0325.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618214.9412.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618216.1026.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618217.2988.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618218.989.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618220.2152.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618221.7188.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618222.9912.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618224.2015.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678669/1777618225.3855.webp"]</t>
         </is>
@@ -2766,39 +3305,64 @@
         </is>
       </c>
       <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr"/>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>4565*1821*1620</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>2780</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr">
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr">
         <is>
           <t>["/uploads/cars/19/1.webp"]</t>
         </is>
       </c>
-      <c r="Y20" t="inlineStr">
+      <c r="AD20" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/05/87678677/1777618147.6141.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678677/1777618148.8913.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678677/1777618150.5032.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678677/1777618151.8114.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678677/1777618152.9066.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678677/1777618154.2208.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678677/1777618155.3543.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678677/1777618156.6699.webp", "https://cn2.pa-server.ru/img/19/2026/05/87678677/1777618157.8062.webp"]</t>
         </is>
@@ -2885,39 +3449,64 @@
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr"/>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>4565*1821*1620</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>2780</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr">
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr">
         <is>
           <t>["/uploads/cars/20/1.webp"]</t>
         </is>
       </c>
-      <c r="Y21" t="inlineStr">
+      <c r="AD21" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/05/87680513/1777618746.3137.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680513/1777618747.1742.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680513/1777618748.0825.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680513/1777618748.9237.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680513/1777618749.9115.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680513/1777618751.1134.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680513/1777618752.1221.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680513/1777618753.1327.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680513/1777618754.1691.webp"]</t>
         </is>
@@ -3004,39 +3593,64 @@
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>(кВт)</t>
-        </is>
-      </c>
+      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>(Н·м)</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr"/>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>(мм)</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>4565*1821*1620</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>2780</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>(л)</t>
-        </is>
-      </c>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr">
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="Y22" t="inlineStr">
+      <c r="AD22" t="inlineStr">
         <is>
           <t>["https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618986.9922.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618988.3693.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618989.5232.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618990.4457.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618991.3594.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618992.1582.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618993.4086.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618994.4797.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618995.489.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618996.4484.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618997.3732.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777618998.9261.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777619000.043.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777619001.0476.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777619002.3094.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777619003.1596.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777619004.4165.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777619005.2651.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777619006.0387.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777619007.3396.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777619008.893.webp", "https://cn2.pa-server.ru/img/19/2026/05/87680952/1777619010.2366.webp"]</t>
         </is>

</xml_diff>

<commit_message>
Add Volkswagen catalog batch
</commit_message>
<xml_diff>
--- a/app/data/korex_latest.xlsx
+++ b/app/data/korex_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF47"/>
+  <dimension ref="A1:AF72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -727,7 +727,7 @@
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>["/uploads/cars/1/1.webp", "/uploads/cars/1/2.webp", "/uploads/cars/1/3.webp"]</t>
+          <t>["/uploads/cars/1/1.webp", "/uploads/cars/1/2.webp", "/uploads/cars/1/3.webp", "/uploads/cars/1/4.webp"]</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -7690,6 +7690,4016 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Volkswagen Tiguan L 2022, пробег 52000 км</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/tiguan-l/1_82894641/</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Tiguan L</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>¥ 113 900</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>9 / 2022</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Tiguan L 
+Volkswagen Tiguan L 2022, пробег 52000 км</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Tiguan L 2023 280TSI Automatic 2WD Trendy Limited Edition</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>6.99</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>6.99</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>4733*1839*1673</t>
+        </is>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>2791</t>
+        </is>
+      </c>
+      <c r="AB48" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AD48" t="inlineStr"/>
+      <c r="AE48" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197682.6262.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197683.7291.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197684.9169.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197686.1804.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197687.1611.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197688.1623.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197689.3196.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197690.4819.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197691.4989.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197692.6788.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197693.6618.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197694.6558.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197696.1895.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197697.3218.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197698.4951.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197699.4781.webp", "https://cn2.pa-server.ru/img/19/2026/04/82894641/1775197700.58.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Volkswagen Tiguan L 2023, пробег 70000 км</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/tiguan-l/1_82896240/</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Tiguan L</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>¥ 171 800</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>3 / 2023</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Tiguan L 
+Volkswagen Tiguan L 2023, пробег 70000 км</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Tiguan L 2023 280TSI Automatic 2WD Trendy Limited Edition</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>6.99</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>6.99</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>4733*1839*1673</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>2791</t>
+        </is>
+      </c>
+      <c r="AB49" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AD49" t="inlineStr"/>
+      <c r="AE49" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF49" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483102.0836.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483103.1251.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483104.2248.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483105.115.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483105.8676.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483106.8219.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483108.0268.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483108.9631.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483109.8097.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483110.8538.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483111.9189.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483112.7248.webp", "https://cn2.pa-server.ru/img/19/2026/04/82896240/1775483113.6151.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Volkswagen Tiguan L 2022, пробег 26000 км</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/tiguan-l/1_84157539/</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Tiguan L</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>¥ 113 900</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>12 / 2022</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Tiguan L 
+Volkswagen Tiguan L 2022, пробег 26000 км</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Tiguan L 2023 280TSI Automatic 2WD Trendy Limited Edition</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>6.99</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>6.99</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>4733*1839*1673</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>2791</t>
+        </is>
+      </c>
+      <c r="AB50" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AD50" t="inlineStr"/>
+      <c r="AE50" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557863.2608.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557864.2365.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557865.4084.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557866.6094.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557867.8299.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557868.7728.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557869.7162.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557870.8989.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557872.1785.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557873.1785.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557874.1654.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557875.3889.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557876.5907.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557877.8074.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557878.8751.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557879.8279.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557881.1532.webp", "https://cn2.pa-server.ru/img/19/2026/04/84157539/1775557882.2143.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Volkswagen Tiguan L 2023, пробег 30000 км</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/tiguan-l/1_86896269/</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Tiguan L</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>¥ 162 000</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>5 / 2023</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Tiguan L 
+Volkswagen Tiguan L 2023, пробег 30000 км</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Tiguan L 2023 280TSI Automatic 2WD Trendy Limited Edition</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>6.99</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>6.99</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>4733*1839*1673</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>2791</t>
+        </is>
+      </c>
+      <c r="AB51" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC51" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AD51" t="inlineStr"/>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262165.2952.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262166.1395.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262168.8407.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262169.5937.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262170.3741.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262172.4898.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262173.4458.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262174.3913.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262175.2641.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262176.365.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262177.6066.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262178.7073.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262180.1336.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262181.4067.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262182.5034.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262183.45.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262184.8563.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262185.6175.webp", "https://cn2.pa-server.ru/img/19/2026/04/86896269/1777262186.389.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Volkswagen Tiguan L 2023, пробег 48000 км</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/tiguan-l/1_87920707/</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Tiguan L</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>¥ 162 000</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>3 / 2023</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Tiguan L 
+Volkswagen Tiguan L 2023, пробег 48000 км</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Tiguan L 2023 280TSI Automatic 2WD Trendy Limited Edition</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>6.99</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>6.99</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>4733*1839*1673</t>
+        </is>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>2791</t>
+        </is>
+      </c>
+      <c r="AB52" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC52" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AD52" t="inlineStr"/>
+      <c r="AE52" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771026.0324.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771027.3958.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771028.7238.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771030.0744.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771031.4372.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771032.508.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771034.2345.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771035.4912.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771036.8136.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771038.7135.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771040.0903.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771041.6116.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771042.7376.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771044.1217.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771046.0878.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771047.4284.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771048.5423.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771049.6829.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771051.1893.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771052.2167.webp", "https://cn2.pa-server.ru/img/19/2026/05/87920707/1777771053.5524.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Volkswagen Tayron 2023, пробег 42000 км</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/tayron/1_66251425/</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Tayron</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>¥ 129 800</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>1 / 2023</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Tayron 
+Volkswagen Tayron 2023, пробег 42000 км</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Tanyue 2023 280TSI 2WD Luxury Plus Advanced Edition</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>FAW-Volkswagen</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>7.08</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>7.08</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>10.6</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>4593*1860*1665</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>2731</t>
+        </is>
+      </c>
+      <c r="AB53" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC53" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AD53" t="inlineStr"/>
+      <c r="AE53" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF53" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197892.836.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197894.836.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197896.2378.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197897.7855.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197899.293.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197901.2167.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197902.6763.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197904.5187.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197906.3175.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197908.0295.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197909.4481.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197910.7454.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197912.1645.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197913.523.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197915.0712.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197916.8002.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197918.4277.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197919.927.webp", "https://cn2.pa-server.ru/img/19/2026/02/66251425/1770197921.3029.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Volkswagen Tayron 2021, пробег 60800 км</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/tayron/1_78025610/</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Tayron</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>¥ 116 800</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>1 / 2021</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Tayron 
+Volkswagen Tayron 2021, пробег 60800 км</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Tanyue 2020 280TSI 2WD Luxury Smart Edition</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>FAW-Volkswagen</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>4589*1860*1660</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>2731</t>
+        </is>
+      </c>
+      <c r="AB54" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AD54" t="inlineStr"/>
+      <c r="AE54" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF54" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246661.8694.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246662.9984.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246664.1808.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246665.6081.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246666.695.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246668.2731.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246669.21.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246670.5106.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246671.8095.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246673.0216.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246674.1928.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246675.3657.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246676.2081.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246677.2215.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246677.9437.webp", "https://cn2.pa-server.ru/img/19/2026/03/78025610/1773246679.2484.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Volkswagen Tayron 2022, пробег 44000 км</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/tayron/1_84698393/</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Tayron</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>¥ 128 000</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>1 / 2022</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Tayron 
+Volkswagen Tayron 2022, пробег 44000 км</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Tanyue 2021 280TSI 2WD Luxury Smart Edition</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>FAW-Volkswagen</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>4589*1860*1660</t>
+        </is>
+      </c>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>2731</t>
+        </is>
+      </c>
+      <c r="AB55" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC55" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AD55" t="inlineStr"/>
+      <c r="AE55" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF55" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803442.9651.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803444.0445.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803444.9353.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803445.9908.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803446.9095.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803447.6722.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803448.676.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803449.8896.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803450.8603.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803451.8993.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803453.1069.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803454.0934.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803454.9192.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803455.8148.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803456.8755.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803457.7265.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803458.6351.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803459.4074.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803460.4604.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698393/1775803461.1683.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Volkswagen Tayron 2022, пробег 34000 км</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/tayron/1_84698395/</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Tayron</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>¥ 129 800</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>1 / 2022</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Tayron 
+Volkswagen Tayron 2022, пробег 34000 км</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Tanyue 2021 280TSI 2WD Luxury Smart Edition</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>FAW-Volkswagen</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>4589*1860*1660</t>
+        </is>
+      </c>
+      <c r="Z56" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>2731</t>
+        </is>
+      </c>
+      <c r="AB56" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC56" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AD56" t="inlineStr"/>
+      <c r="AE56" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF56" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803442.9649.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803443.9491.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803444.9446.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803446.0301.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803447.0125.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803448.0779.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803449.1019.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803449.8925.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803450.7782.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803451.7653.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803452.6126.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803453.4044.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803454.4196.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803455.4756.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803456.4319.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803457.8453.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803459.0944.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803460.0712.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803460.8935.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803461.8082.webp", "https://cn2.pa-server.ru/img/19/2026/04/84698395/1775803462.5427.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Volkswagen Tayron 2022, пробег 62000 км</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/tayron/1_86172281/</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Tayron</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>¥ 129 800</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>4 / 2022</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Tayron 
+Volkswagen Tayron 2022, пробег 62000 км</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Tanyue 2022 280TSI 2WD Luxury Smart Edition</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>FAW-Volkswagen</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>4589*1860*1660</t>
+        </is>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>2731</t>
+        </is>
+      </c>
+      <c r="AB57" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC57" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="AD57" t="inlineStr"/>
+      <c r="AE57" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF57" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617161.9579.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617163.4602.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617164.6625.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617165.7079.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617167.0004.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617168.0469.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617169.0443.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617170.3179.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617171.504.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617172.9442.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617173.9095.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617174.8377.webp", "https://cn2.pa-server.ru/img/19/2026/04/86172281/1776617175.855.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Volkswagen Bora 2021, пробег 40000 км</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/bora/1_78311302/</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Bora</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>¥ 72 100</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2 / 2021</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Bora 
+Volkswagen Bora 2021, пробег 40000 км</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>112 л.с. (82.4 кВт)</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Bora 2021 1.5L Автоматическая Comfort Smart Edition</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>FAW-Volkswagen</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>6.31</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>6.31</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>13.7</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>4663*1815*1462</t>
+        </is>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>2688</t>
+        </is>
+      </c>
+      <c r="AB58" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC58" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AD58" t="inlineStr"/>
+      <c r="AE58" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF58" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/03/78311302/1773397262.6107.webp", "https://cn2.pa-server.ru/img/19/2026/03/78311302/1773397264.1996.webp", "https://cn2.pa-server.ru/img/19/2026/03/78311302/1773397266.2235.webp", "https://cn2.pa-server.ru/img/19/2026/03/78311302/1773397268.0714.webp", "https://cn2.pa-server.ru/img/19/2026/03/78311302/1773397269.8916.webp", "https://cn2.pa-server.ru/img/19/2026/03/78311302/1773397271.2289.webp", "https://cn2.pa-server.ru/img/19/2026/03/78311302/1773397272.2238.webp", "https://cn2.pa-server.ru/img/19/2026/03/78311302/1773397273.7426.webp", "https://cn2.pa-server.ru/img/19/2026/03/78311302/1773397275.1788.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Volkswagen Bora 2023, пробег 36700 км</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/bora/1_86659154/</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Bora</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>¥ 71 800</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>9 / 2023</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Bora 
+Volkswagen Bora 2023, пробег 36700 км</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>1200 см³</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>115 л.с. (84.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Bora 2023 200TSI DSG Joy-Drive PRO Edition</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>FAW-Volkswagen</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>5.78</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>5.78</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>4672*1815*1478</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>1200 см³</t>
+        </is>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>2688</t>
+        </is>
+      </c>
+      <c r="AB59" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC59" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AD59" t="inlineStr"/>
+      <c r="AE59" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF59" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933062.0835.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933063.7756.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933064.7941.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933066.2344.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933067.6649.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933069.4766.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933070.8458.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933071.9436.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933073.3264.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933074.2797.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933075.7857.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933077.0802.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933078.1427.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933079.4253.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933080.3813.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933081.5079.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933083.1293.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933083.8837.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933084.8835.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933085.9562.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933087.0235.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933088.1932.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933089.1608.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933089.918.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933090.8525.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933092.0217.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933092.8326.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933094.3393.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933095.4134.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933096.394.webp", "https://cn2.pa-server.ru/img/19/2026/04/86659154/1776933097.4156.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Volkswagen Bora 2022, пробег 31700 км</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/bora/1_88691957/</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Bora</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>¥ 71 800</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>1 / 2022</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Bora 
+Volkswagen Bora 2022, пробег 31700 км</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>112 л.с. (82.4 кВт)</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Bora 2021 1.5L Автоматическая Comfort Smart Edition</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>FAW-Volkswagen</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>6.31</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>6.31</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>13.7</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>4663*1815*1462</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>2688</t>
+        </is>
+      </c>
+      <c r="AB60" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC60" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AD60" t="inlineStr"/>
+      <c r="AE60" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF60" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071387.785.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071388.7209.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071390.3623.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071391.5331.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071392.1589.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071392.8077.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071393.8559.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071394.865.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071395.7771.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071396.5682.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071397.6794.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071398.9637.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071400.2028.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071401.7559.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071402.8145.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071403.5957.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071404.518.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071405.239.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071406.0576.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071406.7725.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071407.7541.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071408.547.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071409.5904.webp", "https://cn2.pa-server.ru/img/19/2026/05/88691957/1778071410.3361.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Volkswagen Bora 2023, пробег 30000 км</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/bora/1_88692430/</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Bora</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>¥ 71 800</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>5 / 2023</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Bora 
+Volkswagen Bora 2023, пробег 30000 км</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>1200 см³</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>115 л.с. (84.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Bora 2023 200TSI DSG Joy-Drive PRO Edition</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>FAW-Volkswagen</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>5.78</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>5.78</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>4672*1815*1478</t>
+        </is>
+      </c>
+      <c r="Z61" t="inlineStr">
+        <is>
+          <t>1200 см³</t>
+        </is>
+      </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>2688</t>
+        </is>
+      </c>
+      <c r="AB61" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC61" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AD61" t="inlineStr"/>
+      <c r="AE61" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF61" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071567.3706.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071568.5449.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071569.4858.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071570.4154.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071571.389.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071572.717.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071574.0216.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071575.0818.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071576.3656.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071577.6875.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071579.2566.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071580.2776.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071581.4686.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071582.7717.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071584.0187.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071585.4007.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071586.9596.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071588.4374.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071589.5549.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071591.023.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071592.1111.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071593.4877.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692430/1778071594.7064.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Volkswagen Bora 2021, пробег 30000 км</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/bora/1_88692761/</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Bora</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>¥ 72 100</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>6 / 2021</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Bora 
+Volkswagen Bora 2021, пробег 30000 км</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>112 л.с. (82.4 кВт)</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Bora 2021 1.5L Автоматическая модная смарт-версия</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>FAW-Volkswagen</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>6.31</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>6.31</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>13.7</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>4663*1815*1462</t>
+        </is>
+      </c>
+      <c r="Z62" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>2688</t>
+        </is>
+      </c>
+      <c r="AB62" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC62" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="AD62" t="inlineStr"/>
+      <c r="AE62" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF62" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071806.9998.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071808.5401.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071810.5391.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071811.8379.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071812.9871.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071813.9039.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071814.873.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071815.7701.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071816.9916.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071818.2094.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071819.6801.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071820.4904.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071821.5721.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071822.9757.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071824.505.webp", "https://cn2.pa-server.ru/img/19/2026/05/88692761/1778071825.3295.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Volkswagen Lavida 2022, пробег 70000 км</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/lavida/1_79851003/</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Lavida</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>¥ 56 100</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>11 / 2022</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Lavida 
+Volkswagen Lavida 2022, пробег 70000 км</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Lavida 2023 280TSI DSG Starry Sky Edition</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>5.78</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>5.78</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>4678*1806*1474</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>2688</t>
+        </is>
+      </c>
+      <c r="AB63" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC63" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="AD63" t="inlineStr"/>
+      <c r="AE63" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF63" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933961.8829.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933963.2847.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933964.7694.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933966.2399.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933967.5432.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933968.8349.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933970.2496.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933971.2781.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933972.345.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933973.4913.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933974.967.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933976.9977.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933978.3201.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933979.7591.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933981.0972.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933982.4733.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933983.991.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933985.3612.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933986.4259.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933987.7059.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933989.3399.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933991.6295.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933992.8376.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933994.2045.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933995.3116.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933996.3779.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933997.449.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773933999.2421.webp", "https://cn2.pa-server.ru/img/19/2026/03/79851003/1773934000.4224.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Volkswagen Lavida 2022, пробег 33000 км</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/lavida/1_83680865/</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Lavida</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>¥ 56 100</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>12 / 2022</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Lavida 
+Volkswagen Lavida 2022, пробег 33000 км</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>112 л.с. (82.4 кВт)</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Lavida 2023 1.5L Automatic Full-Edge Edition</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>5.92</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>5.92</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>4678*1806*1474</t>
+        </is>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>2688</t>
+        </is>
+      </c>
+      <c r="AB64" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC64" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="AD64" t="inlineStr"/>
+      <c r="AE64" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF64" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394002.0947.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394002.9046.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394003.6722.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394004.4284.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394005.1645.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394005.8867.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394006.6086.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394007.5998.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394008.9391.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394009.7831.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394010.6568.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394011.5921.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394012.6194.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394013.5096.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394014.391.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394015.3093.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394015.9557.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394017.785.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394018.7531.webp", "https://cn2.pa-server.ru/img/19/2026/04/83680865/1775394019.6917.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Volkswagen Lavida 2022, пробег 64200 км</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/lavida/1_84669988/</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Lavida</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>¥ 56 100</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>12 / 2022</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Lavida 
+Volkswagen Lavida 2022, пробег 64200 км</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>112 л.с. (82.4 кВт)</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Lavida 2023 1.5L Automatic Full-Edge Edition</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>5.92</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>5.92</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>4678*1806*1474</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>2688</t>
+        </is>
+      </c>
+      <c r="AB65" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="AD65" t="inlineStr"/>
+      <c r="AE65" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF65" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785382.0217.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785383.0557.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785383.8417.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785385.1467.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785385.9343.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785386.9866.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785388.161.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785389.1428.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785390.2345.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785392.1935.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785393.5797.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785394.8773.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785396.0202.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785397.1168.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785398.3866.webp", "https://cn2.pa-server.ru/img/19/2026/04/84669988/1775785399.4283.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Volkswagen Lavida 2023, пробег 42600 км</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/lavida/1_84671271/</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Lavida</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>¥ 56 000</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>1 / 2023</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Lavida 
+Volkswagen Lavida 2023, пробег 42600 км</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Lavida 2023 280TSI DSG Starry Sky Edition</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>5.78</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>5.78</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X66" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>4678*1806*1474</t>
+        </is>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>2688</t>
+        </is>
+      </c>
+      <c r="AB66" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC66" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="AD66" t="inlineStr"/>
+      <c r="AE66" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF66" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785922.0038.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785923.2876.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785924.4845.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785925.636.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785927.6788.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785928.7225.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785930.3159.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785931.5799.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785933.0889.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785934.5161.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785935.4312.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785936.1938.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785937.2872.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785938.3207.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785939.7509.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785941.0293.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785942.3438.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785943.5217.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785944.8893.webp", "https://cn2.pa-server.ru/img/19/2026/04/84671271/1775785946.3331.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Volkswagen Lavida 2022, пробег 40400 км</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/lavida/1_85157618/</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Lavida</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>¥ 56 100</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>1 / 2022</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Lavida 
+Volkswagen Lavida 2022, пробег 40400 км</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>112 л.с. (82.4 кВт)</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Lavida 2021 1.5L Автоматическая Comfort Edition</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>4670*1806*1474</t>
+        </is>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>1500 см³</t>
+        </is>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>2688</t>
+        </is>
+      </c>
+      <c r="AB67" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC67" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="AD67" t="inlineStr"/>
+      <c r="AE67" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF67" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045302.1999.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045302.9983.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045303.9451.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045304.7698.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045305.5642.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045306.3417.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045307.0826.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045307.9645.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045308.9354.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045309.6674.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045310.5286.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045311.3179.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045312.1887.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045313.0214.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045313.7203.webp", "https://cn2.pa-server.ru/img/19/2026/04/85157618/1776045314.5136.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Volkswagen Passat 2021, пробег 51000 км</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/passat/1_87710922/</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Passat</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>¥ 96 800</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>3 / 2021</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Passat 
+Volkswagen Passat 2021, пробег 51000 км</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Passat 2021 280TSI Элитная версия</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>4933*1836*1469</t>
+        </is>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>2871</t>
+        </is>
+      </c>
+      <c r="AB68" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC68" t="inlineStr">
+        <is>
+          <t>68.5</t>
+        </is>
+      </c>
+      <c r="AD68" t="inlineStr"/>
+      <c r="AE68" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF68" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/05/87710922/1777636385.9617.webp", "https://cn2.pa-server.ru/img/19/2026/05/87710922/1777636387.0897.webp", "https://cn2.pa-server.ru/img/19/2026/05/87710922/1777636388.4063.webp", "https://cn2.pa-server.ru/img/19/2026/05/87710922/1777636389.7043.webp", "https://cn2.pa-server.ru/img/19/2026/05/87710922/1777636391.1443.webp", "https://cn2.pa-server.ru/img/19/2026/05/87710922/1777636392.389.webp", "https://cn2.pa-server.ru/img/19/2026/05/87710922/1777636393.5864.webp", "https://cn2.pa-server.ru/img/19/2026/05/87710922/1777636394.5373.webp", "https://cn2.pa-server.ru/img/19/2026/05/87710922/1777636395.3896.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Volkswagen Passat 2022, пробег 35000 км</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/passat/1_88220352/</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Passat</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>¥ 117 600</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>7 / 2022</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Passat 
+Volkswagen Passat 2022, пробег 35000 км</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Passat 2023 рестайлинг 280TSI Elite Edition</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X69" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>4948*1836*1469</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>2871</t>
+        </is>
+      </c>
+      <c r="AB69" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC69" t="inlineStr">
+        <is>
+          <t>68.5</t>
+        </is>
+      </c>
+      <c r="AD69" t="inlineStr"/>
+      <c r="AE69" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF69" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892587.0809.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892588.3098.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892589.3748.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892591.077.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892593.6019.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892594.8542.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892596.7177.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892597.879.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892598.672.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892599.9239.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892601.0774.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892602.2267.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892603.6286.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892604.5259.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892605.5204.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892606.5732.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892607.8544.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892609.5561.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892610.5819.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892612.0069.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892613.3458.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892614.537.webp", "https://cn2.pa-server.ru/img/19/2026/05/88220352/1777892615.8046.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Volkswagen Passat 2022, пробег 37800 км</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/passat/1_89783276/</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Passat</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>¥ 117 600</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>7 / 2022</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Passat 
+Volkswagen Passat 2022, пробег 37800 км</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Passat 2023 рестайлинг 280TSI Elite Edition</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>4948*1836*1469</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>2871</t>
+        </is>
+      </c>
+      <c r="AB70" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC70" t="inlineStr">
+        <is>
+          <t>68.5</t>
+        </is>
+      </c>
+      <c r="AD70" t="inlineStr"/>
+      <c r="AE70" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF70" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802908.8676.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802910.2344.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802911.4098.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802912.4122.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802913.6658.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802914.5977.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802915.6833.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802916.6423.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802917.8627.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802918.6923.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802919.8589.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802921.3832.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802922.3978.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802924.228.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802926.1901.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802927.5882.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802928.5068.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802929.8712.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783276/1778802931.2037.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Volkswagen Passat 2022, пробег 37000 км</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/passat/1_89783280/</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Passat</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>¥ 117 600</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>7 / 2022</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Passat 
+Volkswagen Passat 2022, пробег 37000 км</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Passat 2023 рестайлинг 280TSI Elite Edition</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>4948*1836*1469</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>2871</t>
+        </is>
+      </c>
+      <c r="AB71" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC71" t="inlineStr">
+        <is>
+          <t>68.5</t>
+        </is>
+      </c>
+      <c r="AD71" t="inlineStr"/>
+      <c r="AE71" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF71" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802908.8765.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802910.3572.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802914.9543.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802917.6957.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802919.3642.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802921.1469.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802922.4535.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802923.8674.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802925.4562.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802926.798.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802928.9107.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802930.4166.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802931.904.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802932.8912.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802934.619.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802936.1416.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802937.7269.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802939.163.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802940.1662.webp", "https://cn2.pa-server.ru/img/19/2026/05/89783280/1778802941.772.webp"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Volkswagen Passat 2022, пробег 48000 км</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://korex-auto.com/china-used/volkswagen/passat/1_89942992/</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Passat</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>¥ 117 600</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>10 / 2022</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Korex 
+Авто из Китая 
+Volkswagen 
+Passat 
+Volkswagen Passat 2022, пробег 48000 км</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>149 л.с. (109.6 кВт)</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>/uploads/fallback.svg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Passat 2023 280TSI Star Elite Edition</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>SAIC Фольксваген</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>Бензин</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Автоматическая коробка передач (АТ)</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Передний привод</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>4948*1836*1469</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>1400 см³</t>
+        </is>
+      </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>2871</t>
+        </is>
+      </c>
+      <c r="AB72" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AC72" t="inlineStr">
+        <is>
+          <t>68.5</t>
+        </is>
+      </c>
+      <c r="AD72" t="inlineStr"/>
+      <c r="AE72" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="AF72" t="inlineStr">
+        <is>
+          <t>["https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934368.2887.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934370.1136.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934371.4369.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934372.4411.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934373.4597.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934374.4748.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934375.5224.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934376.6389.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934377.7408.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934378.7071.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934380.2662.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934381.4779.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934382.474.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934383.7608.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934385.2388.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934386.312.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934387.3516.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934388.4803.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934389.5467.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934390.6469.webp", "https://cn2.pa-server.ru/img/19/2026/05/89942992/1778934391.7648.webp"]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>